<commit_message>
remove fa.vhd from modelsim project
</commit_message>
<xml_diff>
--- a/Documentation/ProjectLog-G12-4645-350-1261.xlsx
+++ b/Documentation/ProjectLog-G12-4645-350-1261.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="55">
   <si>
     <r>
       <rPr>
@@ -413,6 +413,15 @@
     <t xml:space="preserve">Write design topologies megasection: 3.1 RCAN, 3.2 RCAN. Add VHDL code to outline code structure.</t>
   </si>
   <si>
+    <t xml:space="preserve">Do research on how to accurately make estimates about performance. Idea: use estimates based on theoretical circuit structures, and then verify that quartus does not do any drastic restructuring that completely contradicts the theoretical circuit structure.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clean up CSAN, RCAN, code: make them use the same full adder entities. Remove FA.vhd from project. Edit .do scripts to reflect this change. Create new vhdl listing to reflect these changes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Add waveform images, RTL images, VHDL code snippets, and expressions for the design topologies megasection, for use in later parts. </t>
+  </si>
+  <si>
     <r>
       <rPr>
         <sz val="26"/>
@@ -588,7 +597,7 @@
     <numFmt numFmtId="169" formatCode="0.00"/>
     <numFmt numFmtId="170" formatCode="h:mm:ss"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="18">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -708,6 +717,12 @@
       <name val="Times New Roman"/>
       <family val="1"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="6">
@@ -916,7 +931,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="49">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1108,6 +1123,10 @@
     <xf numFmtId="169" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="true"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="4" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -5553,7 +5572,9 @@
         <v>0.999305555555556</v>
       </c>
       <c r="F11" s="33"/>
-      <c r="G11" s="34"/>
+      <c r="G11" s="34" t="s">
+        <v>46</v>
+      </c>
       <c r="H11" s="35" t="n">
         <f aca="false">(E11-D11)*24</f>
         <v>1.98333333333333</v>
@@ -5564,14 +5585,22 @@
       <c r="B12" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="C12" s="30"/>
-      <c r="D12" s="22"/>
-      <c r="E12" s="32"/>
+      <c r="C12" s="30" t="n">
+        <v>46082</v>
+      </c>
+      <c r="D12" s="22" t="n">
+        <v>0.583333333333333</v>
+      </c>
+      <c r="E12" s="32" t="n">
+        <v>0.666666666666667</v>
+      </c>
       <c r="F12" s="33"/>
-      <c r="G12" s="34"/>
+      <c r="G12" s="48" t="s">
+        <v>47</v>
+      </c>
       <c r="H12" s="35" t="n">
         <f aca="false">(E12-D12)*24</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5579,14 +5608,22 @@
       <c r="B13" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="C13" s="30"/>
-      <c r="D13" s="22"/>
-      <c r="E13" s="32"/>
+      <c r="C13" s="30" t="n">
+        <v>46082</v>
+      </c>
+      <c r="D13" s="32" t="n">
+        <v>0.666666666666667</v>
+      </c>
+      <c r="E13" s="32" t="n">
+        <v>0.75</v>
+      </c>
       <c r="F13" s="33"/>
-      <c r="G13" s="34"/>
+      <c r="G13" s="34" t="s">
+        <v>48</v>
+      </c>
       <c r="H13" s="35" t="n">
         <f aca="false">(E13-D13)*24</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5594,14 +5631,20 @@
       <c r="B14" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="C14" s="30"/>
-      <c r="D14" s="22"/>
-      <c r="E14" s="32"/>
+      <c r="C14" s="30" t="n">
+        <v>46082</v>
+      </c>
+      <c r="D14" s="32" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E14" s="32" t="n">
+        <v>0.833333333333333</v>
+      </c>
       <c r="F14" s="33"/>
       <c r="G14" s="34"/>
       <c r="H14" s="35" t="n">
         <f aca="false">(E14-D14)*24</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5609,14 +5652,20 @@
       <c r="B15" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="C15" s="30"/>
-      <c r="D15" s="22"/>
-      <c r="E15" s="32"/>
+      <c r="C15" s="30" t="n">
+        <v>46082</v>
+      </c>
+      <c r="D15" s="32" t="n">
+        <v>0.833333333333333</v>
+      </c>
+      <c r="E15" s="32" t="n">
+        <v>0.916666666666667</v>
+      </c>
       <c r="F15" s="33"/>
       <c r="G15" s="34"/>
       <c r="H15" s="35" t="n">
         <f aca="false">(E15-D15)*24</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5624,14 +5673,20 @@
       <c r="B16" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="C16" s="30"/>
-      <c r="D16" s="22"/>
-      <c r="E16" s="32"/>
+      <c r="C16" s="30" t="n">
+        <v>46082</v>
+      </c>
+      <c r="D16" s="32" t="n">
+        <v>0.916666666666667</v>
+      </c>
+      <c r="E16" s="32" t="n">
+        <v>0.999305555555556</v>
+      </c>
       <c r="F16" s="33"/>
       <c r="G16" s="34"/>
       <c r="H16" s="35" t="n">
         <f aca="false">(E16-D16)*24</f>
-        <v>0</v>
+        <v>1.98333333333333</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6461,7 +6516,7 @@
       <c r="F80" s="46"/>
       <c r="H80" s="47" t="n">
         <f aca="false">SUM(H7:H79)</f>
-        <v>9.98333333333333</v>
+        <v>19.9666666666667</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -7231,7 +7286,7 @@
       <c r="C2" s="6"/>
       <c r="D2" s="6"/>
       <c r="E2" s="7" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="F2" s="7"/>
       <c r="G2" s="7"/>
@@ -7252,7 +7307,7 @@
         <v>5</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C4" s="9"/>
       <c r="D4" s="9"/>
@@ -7265,7 +7320,7 @@
         <v>7</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C5" s="9"/>
       <c r="D5" s="9"/>
@@ -9048,7 +9103,7 @@
       <c r="C2" s="6"/>
       <c r="D2" s="6"/>
       <c r="E2" s="7" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="F2" s="7"/>
       <c r="G2" s="7"/>
@@ -9069,7 +9124,7 @@
         <v>5</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C4" s="9"/>
       <c r="D4" s="9"/>
@@ -9082,7 +9137,7 @@
         <v>7</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C5" s="9"/>
       <c r="D5" s="9"/>
@@ -10847,7 +10902,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="93.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="B1" s="4"/>
       <c r="C1" s="4"/>
@@ -10865,7 +10920,7 @@
       <c r="C2" s="6"/>
       <c r="D2" s="6"/>
       <c r="E2" s="7" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="F2" s="7"/>
       <c r="G2" s="7"/>
@@ -10886,7 +10941,7 @@
         <v>5</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C4" s="9"/>
       <c r="D4" s="9"/>
@@ -10899,7 +10954,7 @@
         <v>7</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C5" s="9"/>
       <c r="D5" s="9"/>

</xml_diff>